<commit_message>
Record optimized 1000-table serving sweep through B8 and refresh comparison workbook
</commit_message>
<xml_diff>
--- a/outputs/01a0735d-f277-7262-b1d0-b87d6db95456/Table OCR latency comparison.xlsx
+++ b/outputs/01a0735d-f277-7262-b1d0-b87d6db95456/Table OCR latency comparison.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency comparison" sheetId="1" r:id="Rbeea867a17e444b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vLLM data" sheetId="2" r:id="R63d4acd3ba8f4549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and notes" sheetId="3" r:id="Ra2f9d677b77e4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency comparison" sheetId="1" r:id="Ra90d21ac51374444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vLLM data" sheetId="2" r:id="Rf58a725d6064474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and notes" sheetId="3" r:id="Ra51333f4e3c9405c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +98,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF92C96F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2EFDA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -210,7 +215,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="61">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -387,6 +392,25 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2298,7 +2322,7 @@
       <x:c r="A28" s="2"/>
       <x:c r="B28" s="2"/>
       <x:c r="C28" s="3" t="str">
-        <x:v>New optimizations · 1,000 requests · 2026-09-05</x:v>
+        <x:v>Latest optimizations · 1,000 requests · 2026-09-06</x:v>
       </x:c>
       <x:c r="D28" s="3" t="str">
         <x:v>New optimizations · 1,000 requests · 2026-09-05</x:v>
@@ -2447,29 +2471,29 @@
     <x:row r="31" ht="24.75" customHeight="1">
       <x:c r="A31" s="2"/>
       <x:c r="B31" s="2"/>
-      <x:c r="C31" s="36" t="str">
+      <x:c r="C31" s="66" t="str">
         <x:v>B1 / C1</x:v>
       </x:c>
-      <x:c r="D31" s="40" t="n">
-        <x:v>0.5726859175631543</x:v>
-      </x:c>
-      <x:c r="E31" s="40" t="n">
-        <x:v>0.3566047759959474</x:v>
-      </x:c>
-      <x:c r="F31" s="40" t="n">
-        <x:v>1.2453623015782798</x:v>
-      </x:c>
-      <x:c r="G31" s="41" t="n">
-        <x:v>1.8107100192282815</x:v>
-      </x:c>
-      <x:c r="H31" s="40" t="n">
-        <x:v>3.69978321625269</x:v>
-      </x:c>
-      <x:c r="I31" s="40" t="n">
-        <x:v>5.059540969901718</x:v>
-      </x:c>
-      <x:c r="J31" s="41" t="n">
-        <x:v>1.7451399089059154</x:v>
+      <x:c r="D31" s="68" t="n">
+        <x:v>0.5213162477005971</x:v>
+      </x:c>
+      <x:c r="E31" s="68" t="n">
+        <x:v>0.33059578901156783</x:v>
+      </x:c>
+      <x:c r="F31" s="68" t="n">
+        <x:v>1.1335126296267846</x:v>
+      </x:c>
+      <x:c r="G31" s="69" t="n">
+        <x:v>1.6565518201270606</x:v>
+      </x:c>
+      <x:c r="H31" s="68" t="n">
+        <x:v>3.3628204637719317</x:v>
+      </x:c>
+      <x:c r="I31" s="68" t="n">
+        <x:v>3.429513827082701</x:v>
+      </x:c>
+      <x:c r="J31" s="69" t="n">
+        <x:v>1.916940128951687</x:v>
       </x:c>
       <x:c r="K31" s="2"/>
       <x:c r="L31" s="49" t="str">
@@ -2519,29 +2543,29 @@
     <x:row r="32" ht="24.75" customHeight="1">
       <x:c r="A32" s="2"/>
       <x:c r="B32" s="2"/>
-      <x:c r="C32" s="36" t="str">
+      <x:c r="C32" s="66" t="str">
         <x:v>B2 / C2</x:v>
       </x:c>
-      <x:c r="D32" s="40" t="n">
-        <x:v>0.6741275758377742</x:v>
-      </x:c>
-      <x:c r="E32" s="40" t="n">
-        <x:v>0.4114297530031763</x:v>
-      </x:c>
-      <x:c r="F32" s="40" t="n">
-        <x:v>1.528275076032151</x:v>
-      </x:c>
-      <x:c r="G32" s="41" t="n">
-        <x:v>2.182853424537461</x:v>
-      </x:c>
-      <x:c r="H32" s="40" t="n">
-        <x:v>4.434693658559118</x:v>
-      </x:c>
-      <x:c r="I32" s="40" t="n">
-        <x:v>4.683510718983598</x:v>
-      </x:c>
-      <x:c r="J32" s="41" t="n">
-        <x:v>2.9597911819339586</x:v>
+      <x:c r="D32" s="68" t="n">
+        <x:v>0.6041275005427887</x:v>
+      </x:c>
+      <x:c r="E32" s="68" t="n">
+        <x:v>0.3743322269874625</x:v>
+      </x:c>
+      <x:c r="F32" s="68" t="n">
+        <x:v>1.336234595521819</x:v>
+      </x:c>
+      <x:c r="G32" s="69" t="n">
+        <x:v>1.9527289563324304</x:v>
+      </x:c>
+      <x:c r="H32" s="68" t="n">
+        <x:v>3.896921452964889</x:v>
+      </x:c>
+      <x:c r="I32" s="68" t="n">
+        <x:v>4.195354482973926</x:v>
+      </x:c>
+      <x:c r="J32" s="69" t="n">
+        <x:v>3.3022555894193437</x:v>
       </x:c>
       <x:c r="K32" s="2"/>
       <x:c r="L32" s="49" t="str">
@@ -2591,29 +2615,29 @@
     <x:row r="33" ht="24.75" customHeight="1">
       <x:c r="A33" s="2"/>
       <x:c r="B33" s="2"/>
-      <x:c r="C33" s="36" t="str">
-        <x:v>B4 / C3</x:v>
-      </x:c>
-      <x:c r="D33" s="40" t="n">
-        <x:v>0.7867940118489787</x:v>
-      </x:c>
-      <x:c r="E33" s="40" t="n">
-        <x:v>0.48407740256516263</x:v>
-      </x:c>
-      <x:c r="F33" s="40" t="n">
-        <x:v>1.7399584487662665</x:v>
-      </x:c>
-      <x:c r="G33" s="41" t="n">
-        <x:v>2.622647292126202</x:v>
-      </x:c>
-      <x:c r="H33" s="40" t="n">
-        <x:v>5.278963240978774</x:v>
-      </x:c>
-      <x:c r="I33" s="40" t="n">
-        <x:v>6.043582064914517</x:v>
-      </x:c>
-      <x:c r="J33" s="41" t="n">
-        <x:v>3.797314857325923</x:v>
+      <x:c r="C33" s="66" t="str">
+        <x:v>B3 / C3</x:v>
+      </x:c>
+      <x:c r="D33" s="68" t="n">
+        <x:v>0.7598435960153583</x:v>
+      </x:c>
+      <x:c r="E33" s="68" t="n">
+        <x:v>0.4687598364544101</x:v>
+      </x:c>
+      <x:c r="F33" s="68" t="n">
+        <x:v>1.713730762887281</x:v>
+      </x:c>
+      <x:c r="G33" s="69" t="n">
+        <x:v>2.4720755729300423</x:v>
+      </x:c>
+      <x:c r="H33" s="68" t="n">
+        <x:v>5.063775968842673</x:v>
+      </x:c>
+      <x:c r="I33" s="68" t="n">
+        <x:v>5.5475653250468895</x:v>
+      </x:c>
+      <x:c r="J33" s="69" t="n">
+        <x:v>3.930970276679353</x:v>
       </x:c>
       <x:c r="K33" s="2"/>
       <x:c r="L33" s="2"/>
@@ -2635,33 +2659,33 @@
     <x:row r="34" ht="24.75" customHeight="1">
       <x:c r="A34" s="2"/>
       <x:c r="B34" s="2"/>
-      <x:c r="C34" s="36" t="str">
+      <x:c r="C34" s="66" t="str">
         <x:v>B4 / C4</x:v>
       </x:c>
-      <x:c r="D34" s="40" t="n">
-        <x:v>0.850941418405855</x:v>
-      </x:c>
-      <x:c r="E34" s="40" t="n">
-        <x:v>0.5118363889632747</x:v>
-      </x:c>
-      <x:c r="F34" s="40" t="n">
-        <x:v>1.962066580797546</x:v>
-      </x:c>
-      <x:c r="G34" s="41" t="n">
-        <x:v>2.790147225355028</x:v>
-      </x:c>
-      <x:c r="H34" s="40" t="n">
-        <x:v>5.694143164759734</x:v>
-      </x:c>
-      <x:c r="I34" s="40" t="n">
-        <x:v>6.40279202000238</x:v>
-      </x:c>
-      <x:c r="J34" s="41" t="n">
-        <x:v>4.673750941937389</x:v>
+      <x:c r="D34" s="68" t="n">
+        <x:v>0.7755472345288145</x:v>
+      </x:c>
+      <x:c r="E34" s="68" t="n">
+        <x:v>0.4701226999750361</x:v>
+      </x:c>
+      <x:c r="F34" s="68" t="n">
+        <x:v>1.7669590109726416</x:v>
+      </x:c>
+      <x:c r="G34" s="69" t="n">
+        <x:v>2.540035831264684</x:v>
+      </x:c>
+      <x:c r="H34" s="68" t="n">
+        <x:v>5.108939005434513</x:v>
+      </x:c>
+      <x:c r="I34" s="68" t="n">
+        <x:v>5.611563332029618</x:v>
+      </x:c>
+      <x:c r="J34" s="69" t="n">
+        <x:v>5.128103389079862</x:v>
       </x:c>
       <x:c r="K34" s="2"/>
       <x:c r="L34" s="49" t="str">
-        <x:v>Ordinary decoding only. Latest CPU preparation and vision padding optimizations; unchanged model, input pixel policy, greedy selection, native vocabulary map, KV4096 and stopping rules.</x:v>
+        <x:v>Ordinary decoding. Packed MLP, complete-layer prefetch, RoPE lookup, linear vision patch projection, vision padding, setup GC freeze and no optional decode timing events. Unchanged input policy, native vocabulary map and KV4096.</x:v>
       </x:c>
       <x:c r="M34" s="49" t="str">
         <x:v>Ordinary decoding only. Latest CPU preparation and vision padding optimizations; unchanged model, input pixel policy, greedy selection, native vocabulary map, KV4096 and stopping rules.</x:v>
@@ -2707,29 +2731,29 @@
     <x:row r="35" ht="24.75" customHeight="1">
       <x:c r="A35" s="2"/>
       <x:c r="B35" s="2"/>
-      <x:c r="C35" s="36" t="str">
-        <x:v>B8 / C8</x:v>
-      </x:c>
-      <x:c r="D35" s="40" t="n">
-        <x:v>1.2322152753287228</x:v>
-      </x:c>
-      <x:c r="E35" s="40" t="n">
-        <x:v>0.7186776890303008</x:v>
-      </x:c>
-      <x:c r="F35" s="40" t="n">
-        <x:v>2.821711886639242</x:v>
-      </x:c>
-      <x:c r="G35" s="41" t="n">
-        <x:v>4.142976103140971</x:v>
-      </x:c>
-      <x:c r="H35" s="40" t="n">
-        <x:v>8.466388167063705</x:v>
-      </x:c>
-      <x:c r="I35" s="40" t="n">
-        <x:v>9.357020128984004</x:v>
-      </x:c>
-      <x:c r="J35" s="41" t="n">
-        <x:v>6.371464571114747</x:v>
+      <x:c r="C35" s="66" t="str">
+        <x:v>B5 / C5</x:v>
+      </x:c>
+      <x:c r="D35" s="68" t="n">
+        <x:v>0.8845392211870058</x:v>
+      </x:c>
+      <x:c r="E35" s="68" t="n">
+        <x:v>0.5350188484298997</x:v>
+      </x:c>
+      <x:c r="F35" s="68" t="n">
+        <x:v>2.0663810262689366</x:v>
+      </x:c>
+      <x:c r="G35" s="69" t="n">
+        <x:v>2.8849450394802245</x:v>
+      </x:c>
+      <x:c r="H35" s="68" t="n">
+        <x:v>5.887338578747585</x:v>
+      </x:c>
+      <x:c r="I35" s="68" t="n">
+        <x:v>6.7386838279198855</x:v>
+      </x:c>
+      <x:c r="J35" s="69" t="n">
+        <x:v>5.605123315729733</x:v>
       </x:c>
       <x:c r="K35" s="2"/>
       <x:c r="L35" s="49" t="str">
@@ -2779,29 +2803,29 @@
     <x:row r="36" ht="24.75" customHeight="1">
       <x:c r="A36" s="2"/>
       <x:c r="B36" s="2"/>
-      <x:c r="C36" s="36" t="str">
-        <x:v>B16 / C16</x:v>
-      </x:c>
-      <x:c r="D36" s="40" t="n">
-        <x:v>1.9334103902485222</x:v>
-      </x:c>
-      <x:c r="E36" s="40" t="n">
-        <x:v>1.1220657555386424</x:v>
-      </x:c>
-      <x:c r="F36" s="40" t="n">
-        <x:v>4.5105511834844965</x:v>
-      </x:c>
-      <x:c r="G36" s="41" t="n">
-        <x:v>6.435093457967739</x:v>
-      </x:c>
-      <x:c r="H36" s="40" t="n">
-        <x:v>13.822808395529865</x:v>
-      </x:c>
-      <x:c r="I36" s="40" t="n">
-        <x:v>15.154038943932392</x:v>
-      </x:c>
-      <x:c r="J36" s="41" t="n">
-        <x:v>7.957404647288651</x:v>
+      <x:c r="C36" s="66" t="str">
+        <x:v>B6 / C6</x:v>
+      </x:c>
+      <x:c r="D36" s="68" t="n">
+        <x:v>0.9974676761954324</x:v>
+      </x:c>
+      <x:c r="E36" s="68" t="n">
+        <x:v>0.5958280664635822</x:v>
+      </x:c>
+      <x:c r="F36" s="68" t="n">
+        <x:v>2.2713731546071365</x:v>
+      </x:c>
+      <x:c r="G36" s="69" t="n">
+        <x:v>3.2565520662174055</x:v>
+      </x:c>
+      <x:c r="H36" s="68" t="n">
+        <x:v>6.556477977633474</x:v>
+      </x:c>
+      <x:c r="I36" s="68" t="n">
+        <x:v>7.884030124987476</x:v>
+      </x:c>
+      <x:c r="J36" s="69" t="n">
+        <x:v>5.942513646912682</x:v>
       </x:c>
       <x:c r="K36" s="2"/>
       <x:c r="L36" s="49" t="str">
@@ -2848,17 +2872,33 @@
       </x:c>
       <x:c r="Z36" s="2"/>
     </x:row>
-    <x:row r="37" ht="23.25" customHeight="1">
+    <x:row r="37" ht="24.75" customHeight="1">
       <x:c r="A37" s="2"/>
       <x:c r="B37" s="2"/>
-      <x:c r="C37" s="2"/>
-      <x:c r="D37" s="2"/>
-      <x:c r="E37" s="2"/>
-      <x:c r="F37" s="2"/>
-      <x:c r="G37" s="2"/>
-      <x:c r="H37" s="2"/>
-      <x:c r="I37" s="2"/>
-      <x:c r="J37" s="2"/>
+      <x:c r="C37" s="66" t="str">
+        <x:v>B7 / C7</x:v>
+      </x:c>
+      <x:c r="D37" s="68" t="n">
+        <x:v>1.0593258181991987</x:v>
+      </x:c>
+      <x:c r="E37" s="68" t="n">
+        <x:v>0.617943222518079</x:v>
+      </x:c>
+      <x:c r="F37" s="68" t="n">
+        <x:v>2.407472352520563</x:v>
+      </x:c>
+      <x:c r="G37" s="69" t="n">
+        <x:v>3.471485421829855</x:v>
+      </x:c>
+      <x:c r="H37" s="68" t="n">
+        <x:v>7.015740477233191</x:v>
+      </x:c>
+      <x:c r="I37" s="68" t="n">
+        <x:v>8.021164715057239</x:v>
+      </x:c>
+      <x:c r="J37" s="69" t="n">
+        <x:v>6.508119820258158</x:v>
+      </x:c>
       <x:c r="K37" s="2"/>
       <x:c r="L37" s="2"/>
       <x:c r="M37" s="2"/>
@@ -2876,36 +2916,36 @@
       <x:c r="Y37" s="2"/>
       <x:c r="Z37" s="2"/>
     </x:row>
-    <x:row r="38" ht="23.25" customHeight="1">
+    <x:row r="38" ht="24.75" customHeight="1">
       <x:c r="A38" s="2"/>
       <x:c r="B38" s="2"/>
-      <x:c r="C38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="D38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="E38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="F38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="G38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="H38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="I38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="J38" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      <x:c r="C38" s="66" t="str">
+        <x:v>B8 / C7</x:v>
+      </x:c>
+      <x:c r="D38" s="68" t="n">
+        <x:v>1.0653884073762456</x:v>
+      </x:c>
+      <x:c r="E38" s="68" t="n">
+        <x:v>0.6112742489785887</x:v>
+      </x:c>
+      <x:c r="F38" s="68" t="n">
+        <x:v>2.393488236877602</x:v>
+      </x:c>
+      <x:c r="G38" s="69" t="n">
+        <x:v>3.582552019687135</x:v>
+      </x:c>
+      <x:c r="H38" s="68" t="n">
+        <x:v>7.117921280496519</x:v>
+      </x:c>
+      <x:c r="I38" s="68" t="n">
+        <x:v>7.991954467957839</x:v>
+      </x:c>
+      <x:c r="J38" s="69" t="n">
+        <x:v>6.468149539254828</x:v>
       </x:c>
       <x:c r="K38" s="2"/>
       <x:c r="L38" s="49" t="str">
-        <x:v>KV4096 limit stops, retained in every latency denominator: B1: 12; B2: 12; B4C3: 12; B4C4: 12; B8: 12; B16: 12. QPS counts returned requests, including these capped outputs; not proof of complete-output goal validation.</x:v>
+        <x:v>Each selected run: 1,000 responses, 988 EOS completions, 12 unchanged KV4096-cap outputs, no request errors. All 1,000 are included in latency and QPS. One physical 910B2 (NPU6), with exclusive ownership verified during measurement.</x:v>
       </x:c>
       <x:c r="M38" s="49" t="str">
         <x:v>KV4096 limit stops, retained in every latency denominator: B1: 12; B2: 12; B4C3: 12; B4C4: 12; B8: 12; B16: 12. QPS counts returned requests, including these capped outputs; not proof of complete-output goal validation.</x:v>
@@ -2948,32 +2988,32 @@
       </x:c>
       <x:c r="Z38" s="2"/>
     </x:row>
-    <x:row r="39" ht="23.25" customHeight="1">
+    <x:row r="39" ht="24.75" customHeight="1">
       <x:c r="A39" s="2"/>
       <x:c r="B39" s="2"/>
-      <x:c r="C39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="D39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="E39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="F39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="G39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="H39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="I39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
-      </x:c>
-      <x:c r="J39" s="29" t="str">
-        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      <x:c r="C39" s="66" t="str">
+        <x:v>B8 / C8</x:v>
+      </x:c>
+      <x:c r="D39" s="68" t="n">
+        <x:v>1.1240035916685593</x:v>
+      </x:c>
+      <x:c r="E39" s="68" t="n">
+        <x:v>0.6648684749961831</x:v>
+      </x:c>
+      <x:c r="F39" s="68" t="n">
+        <x:v>2.5825716336607005</x:v>
+      </x:c>
+      <x:c r="G39" s="69" t="n">
+        <x:v>3.7681284833292006</x:v>
+      </x:c>
+      <x:c r="H39" s="68" t="n">
+        <x:v>7.67259384816396</x:v>
+      </x:c>
+      <x:c r="I39" s="68" t="n">
+        <x:v>8.543899290030822</x:v>
+      </x:c>
+      <x:c r="J39" s="69" t="n">
+        <x:v>6.985774628299913</x:v>
       </x:c>
       <x:c r="K39" s="2"/>
       <x:c r="L39" s="49" t="str">
@@ -3079,14 +3119,30 @@
     <x:row r="41" ht="23.25" customHeight="1">
       <x:c r="A41" s="2"/>
       <x:c r="B41" s="2"/>
-      <x:c r="C41" s="2"/>
-      <x:c r="D41" s="2"/>
-      <x:c r="E41" s="2"/>
-      <x:c r="F41" s="2"/>
-      <x:c r="G41" s="2"/>
-      <x:c r="H41" s="2"/>
-      <x:c r="I41" s="2"/>
-      <x:c r="J41" s="2"/>
+      <x:c r="C41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="D41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="E41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="F41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="G41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="H41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="I41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="J41" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
       <x:c r="K41" s="2"/>
       <x:c r="L41" s="2"/>
       <x:c r="M41" s="2"/>
@@ -3103,6 +3159,84 @@
       <x:c r="X41" s="2"/>
       <x:c r="Y41" s="2"/>
       <x:c r="Z41" s="2"/>
+    </x:row>
+    <x:row r="42" ht="23.25" customHeight="1">
+      <x:c r="C42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="D42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="E42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="F42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="G42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="H42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="I42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+      <x:c r="J42" s="29" t="str">
+        <x:v>Seed 3: all 665 tables once, then 335 distinct tables from the same corpus. Identical order in every lane. B = static decode batch; C = maximum requests in flight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="23.25" customHeight="1">
+      <x:c r="C44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="D44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="E44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="F44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="G44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="H44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="I44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="J44" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="23.25" customHeight="1">
+      <x:c r="C45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="D45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="E45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="F45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="G45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="H45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="I45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
+      <x:c r="J45" s="29" t="str">
+        <x:v>One new 1,000-request run per tested configuration. B2 shows the higher-P95 run of all three validations (the new reconfirmation). B5 retains the higher-P95 run of its two earlier validations. All metrics in each row come from one run.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3124,10 +3258,11 @@
     <x:mergeCell ref="C25:Y25"/>
     <x:mergeCell ref="C28:J28"/>
     <x:mergeCell ref="C29:E29"/>
-    <x:mergeCell ref="C38:J39"/>
     <x:mergeCell ref="L30:Y32"/>
     <x:mergeCell ref="L34:Y36"/>
     <x:mergeCell ref="L38:Y40"/>
+    <x:mergeCell ref="C41:J42"/>
+    <x:mergeCell ref="C44:J45"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="M6:O6">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -3754,12 +3889,12 @@
         <x:v>Ratios use the photo-displayed, rounded values for both engines. Mean and P95 = vLLM / custom; QPS = custom / vLLM. Values above 1× favor custom. Full-precision vLLM measurements remain in the data tab.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="45" customHeight="1">
+    <x:row r="9" ht="71.25" customHeight="1">
       <x:c r="A9" s="57" t="str">
         <x:v>New comparison</x:v>
       </x:c>
       <x:c r="B9" s="58" t="str">
-        <x:v>table_1000_matrix_02fe5645_20260905. Fixed seed 3; 1,000 submissions per lane, 665 unique crops. Full HTTP submission-to-response timing; payload preparation, model startup and full-request warmup outside timing.</x:v>
+        <x:v>Current sweep: table_optimized_c1_to_c7_9f6e486d_20260906, each lane's measured summary. B2 uses the new reconfirmation (highest P95 of three). B5: table_packed_noevents_b5c5_b0f1cac7_20260906/validation1000_a (higher P95 of two). Same seed-3 sequence. B8/C7 and B8/C8 share a warmed server, with a separate complete-request warmup before each run.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Record optimized B16 C16 1000-table validation and append spreadsheet result
</commit_message>
<xml_diff>
--- a/outputs/01a0735d-f277-7262-b1d0-b87d6db95456/Table OCR latency comparison.xlsx
+++ b/outputs/01a0735d-f277-7262-b1d0-b87d6db95456/Table OCR latency comparison.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency comparison" sheetId="1" r:id="Ra90d21ac51374444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vLLM data" sheetId="2" r:id="Rf58a725d6064474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and notes" sheetId="3" r:id="Ra51333f4e3c9405c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency comparison" sheetId="1" r:id="Rbc9fb4a729854d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vLLM data" sheetId="2" r:id="R28e4ab6dde504911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources and notes" sheetId="3" r:id="R123ea1b4b2744ba7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -73,7 +73,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +98,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF92C96F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2EFDA"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -215,7 +220,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="70">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -410,6 +415,21 @@
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -3060,17 +3080,33 @@
       </x:c>
       <x:c r="Z39" s="2"/>
     </x:row>
-    <x:row r="40" ht="23.25" customHeight="1">
+    <x:row r="40" ht="24.75" customHeight="1">
       <x:c r="A40" s="2"/>
       <x:c r="B40" s="2"/>
-      <x:c r="C40" s="2"/>
-      <x:c r="D40" s="2"/>
-      <x:c r="E40" s="2"/>
-      <x:c r="F40" s="2"/>
-      <x:c r="G40" s="2"/>
-      <x:c r="H40" s="2"/>
-      <x:c r="I40" s="2"/>
-      <x:c r="J40" s="2"/>
+      <x:c r="C40" s="71" t="str">
+        <x:v>B16 / C16</x:v>
+      </x:c>
+      <x:c r="D40" s="73" t="n">
+        <x:v>1.8402280153116444</x:v>
+      </x:c>
+      <x:c r="E40" s="73" t="n">
+        <x:v>1.053500725014601</x:v>
+      </x:c>
+      <x:c r="F40" s="73" t="n">
+        <x:v>4.320971092197579</x:v>
+      </x:c>
+      <x:c r="G40" s="74" t="n">
+        <x:v>6.105224792403168</x:v>
+      </x:c>
+      <x:c r="H40" s="73" t="n">
+        <x:v>13.219456814958248</x:v>
+      </x:c>
+      <x:c r="I40" s="73" t="n">
+        <x:v>14.079549701069482</x:v>
+      </x:c>
+      <x:c r="J40" s="74" t="n">
+        <x:v>8.364789333155967</x:v>
+      </x:c>
       <x:c r="K40" s="2"/>
       <x:c r="L40" s="49" t="str">
         <x:v>KV4096 limit stops, retained in every latency denominator: B1: 12; B2: 12; B4C3: 12; B4C4: 12; B8: 12; B16: 12. QPS counts returned requests, including these capped outputs; not proof of complete-output goal validation.</x:v>

</xml_diff>